<commit_message>
Update README.md to specify required columns for excel data files and correct output folder path
</commit_message>
<xml_diff>
--- a/tests/testthat/test_data/general_info_test.xlsx
+++ b/tests/testthat/test_data/general_info_test.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kise-my.sharepoint.com/personal/felix_falk_ki_se/Documents/Skrivbordet/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kise-my.sharepoint.com/personal/felix_falk_ki_se/Documents/Dokument/nmdsg14bFigures/tests/testthat/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{B7534E70-E8C5-4144-90BC-81577A7B56FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1120" yWindow="660" windowWidth="28240" windowHeight="16660" xr2:uid="{1ACEF37F-179E-B74C-97F3-FE4E441611A6}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="24000" xr2:uid="{1ACEF37F-179E-B74C-97F3-FE4E441611A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -904,5 +904,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>